<commit_message>
feat: monster, TrainData 불러오기 성공
</commit_message>
<xml_diff>
--- a/Assets/TrainDefenseData.xlsx
+++ b/Assets/TrainDefenseData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <bookViews>
-    <workbookView xWindow="5415" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1"/>
+    <workbookView xWindow="5415" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Monster_Data" sheetId="1" r:id="rId1"/>
@@ -35,16 +35,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="38">
   <si>
     <t xml:space="preserve">id</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">name</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve">description</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -85,14 +81,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">Normal Monster</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">Simple Normal Monster</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve">attack_damage</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -105,22 +93,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">메인 기차</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">메인 기차는 모든 기차에 기본이 되는 기차이다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">기관총 포탑</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">빠른 속도로 적을 공격 한다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve">미사일 포탑</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -137,18 +109,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">냉기 포탑</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve">충격 포탑</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t xml:space="preserve">범위 내에 있는 적들을 느리게 하고 지속 피해를 준다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve">범위 내에 있는 적들을 밀치고 피해를 준다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -190,6 +154,21 @@
   </si>
   <si>
     <t xml:space="preserve">Turret</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.5</t>
   </si>
 </sst>
 </file>
@@ -573,75 +552,75 @@
         <v>0</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="F1" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="0" t="s">
+      <c r="G1" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="H1" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="I1" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="J1" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="0" t="s">
+      <c r="K1" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="L1" s="0" t="s">
         <v>10</v>
-      </c>
-      <c r="L1" s="0" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.55">
       <c r="A2" s="0" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="D2" s="0">
-        <v>20</v>
-      </c>
-      <c r="E2" s="0">
-        <v>2</v>
-      </c>
-      <c r="F2" s="0">
-        <v>6</v>
-      </c>
-      <c r="G2" s="0">
-        <v>1</v>
-      </c>
-      <c r="H2" s="0">
-        <v>10</v>
-      </c>
-      <c r="I2" s="0">
-        <v>15</v>
-      </c>
-      <c r="J2" s="0">
-        <v>5</v>
-      </c>
-      <c r="K2" s="0">
-        <v>7</v>
-      </c>
-      <c r="L2" s="0">
-        <v>5</v>
+        <v>23</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="L2" s="0" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -653,7 +632,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="2" width="15.640625" customWidth="1"/>
@@ -661,31 +640,37 @@
     <col min="4" max="13" width="15.640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A2" s="0" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="0" t="b">
+        <v>28</v>
+      </c>
+      <c r="D2" s="0">
+        <v>100</v>
+      </c>
+      <c r="E2" s="0" t="b">
         <v>0</v>
       </c>
     </row>
@@ -698,7 +683,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="2" width="15.640625" customWidth="1"/>
@@ -706,107 +691,119 @@
     <col min="4" max="13" width="15.640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.55">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.55">
+      <c r="A2" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="0">
+        <v>100</v>
+      </c>
+      <c r="E2" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="F2" s="0">
+        <v>5</v>
+      </c>
+      <c r="G2" s="0">
+        <v>10</v>
+      </c>
+      <c r="H2" s="0">
+        <v>1</v>
+      </c>
+      <c r="I2" s="0">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="E1" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G1" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H1" s="0" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.55">
-      <c r="A2" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>41</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="E2" s="0">
-        <v>5</v>
-      </c>
-      <c r="F2" s="0">
-        <v>3</v>
-      </c>
-      <c r="G2" s="0">
-        <v>1</v>
-      </c>
-      <c r="H2" s="0">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.55">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A3" s="0">
         <v>30002</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="D3" s="0">
         <v>100</v>
       </c>
       <c r="E3" s="0">
+        <v>100</v>
+      </c>
+      <c r="F3" s="0">
         <v>5</v>
       </c>
-      <c r="F3" s="0">
-        <v>1</v>
-      </c>
       <c r="G3" s="0">
         <v>1</v>
       </c>
       <c r="H3" s="0">
+        <v>1</v>
+      </c>
+      <c r="I3" s="0">
         <v>0.2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.55">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A4" s="0">
         <v>30003</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D4" s="0">
         <v>100</v>
       </c>
       <c r="E4" s="0">
+        <v>100</v>
+      </c>
+      <c r="F4" s="0">
         <v>10</v>
       </c>
-      <c r="F4" s="0">
+      <c r="G4" s="0">
         <v>5</v>
       </c>
-      <c r="G4" s="0">
-        <v>1</v>
-      </c>
       <c r="H4" s="0">
+        <v>1</v>
+      </c>
+      <c r="I4" s="0">
         <v>1</v>
       </c>
     </row>
@@ -818,7 +815,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="2" width="15.640625" customWidth="1"/>
@@ -826,81 +823,90 @@
     <col min="4" max="13" width="15.640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.55">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.55">
+      <c r="A2" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="0">
+        <v>100</v>
+      </c>
+      <c r="E2" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="F2" s="0">
+        <v>5</v>
+      </c>
+      <c r="G2" s="0">
+        <v>10</v>
+      </c>
+      <c r="H2" s="0">
+        <v>1</v>
+      </c>
+      <c r="I2" s="0">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="E1" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="G1" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="H1" s="0" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.55">
-      <c r="A2" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="E2" s="0">
-        <v>5</v>
-      </c>
-      <c r="F2" s="0">
-        <v>1</v>
-      </c>
-      <c r="G2" s="0">
-        <v>1</v>
-      </c>
-      <c r="H2" s="0">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.55">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A3" s="0">
         <v>40002</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="D3" s="0">
         <v>100</v>
       </c>
-      <c r="E3" s="0">
+      <c r="E3" s="0" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" s="0">
         <v>5</v>
       </c>
-      <c r="F3" s="0">
-        <v>1</v>
-      </c>
       <c r="G3" s="0">
         <v>1</v>
       </c>
       <c r="H3" s="0">
+        <v>1</v>
+      </c>
+      <c r="I3" s="0">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: stageData 잘 불러와짐, TrichoiceDB Db로 통합
</commit_message>
<xml_diff>
--- a/Assets/TrainDefenseData.xlsx
+++ b/Assets/TrainDefenseData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <bookViews>
-    <workbookView xWindow="5415" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="3"/>
+    <workbookView xWindow="7680" yWindow="-15555" windowWidth="16605" windowHeight="10845" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Monster_Data" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="36">
   <si>
     <t xml:space="preserve">id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -120,55 +120,53 @@
     <t xml:space="preserve">monster_name</t>
   </si>
   <si>
-    <t xml:space="preserve">slime_01</t>
+    <t xml:space="preserve">basic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">train_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">is_main_train</t>
+  </si>
+  <si>
+    <t xml:space="preserve">desc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stage_inspection_time</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Basic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t xml:space="preserve">Slime</t>
-  </si>
-  <si>
-    <t xml:space="preserve">basic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">train_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">is_main_train</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">stage_end_time</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">10;20;30</t>
   </si>
   <si>
     <t xml:space="preserve">train_basic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Basic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">desc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">range_basic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Range</t>
-  </si>
-  <si>
-    <t xml:space="preserve">turret_basic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Turret</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.5</t>
   </si>
 </sst>
 </file>
@@ -586,41 +584,41 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.55">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="0">
+        <v>10001</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>23</v>
-      </c>
       <c r="D2" s="0" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H2" s="0" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="J2" s="0" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="K2" s="0" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="L2" s="0" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -645,7 +643,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>1</v>
@@ -654,18 +652,18 @@
         <v>3</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A2" s="0" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D2" s="0">
         <v>100</v>
@@ -683,7 +681,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="2" width="15.640625" customWidth="1"/>
@@ -696,7 +694,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>1</v>
@@ -705,7 +703,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F1" s="0" t="s">
         <v>10</v>
@@ -721,32 +719,32 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55">
-      <c r="A2" s="0" t="s">
-        <v>31</v>
+      <c r="A2" s="0">
+        <v>30001</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="D2" s="0">
         <v>100</v>
       </c>
-      <c r="E2" s="0" t="b">
-        <v>0</v>
+      <c r="E2" s="0">
+        <v>100</v>
       </c>
       <c r="F2" s="0">
         <v>5</v>
       </c>
       <c r="G2" s="0">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H2" s="0">
         <v>1</v>
       </c>
       <c r="I2" s="0">
-        <v>2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.55">
@@ -754,10 +752,10 @@
         <v>30002</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C3" s="0" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" s="0">
         <v>100</v>
@@ -766,44 +764,15 @@
         <v>100</v>
       </c>
       <c r="F3" s="0">
+        <v>10</v>
+      </c>
+      <c r="G3" s="0">
         <v>5</v>
       </c>
-      <c r="G3" s="0">
-        <v>1</v>
-      </c>
       <c r="H3" s="0">
         <v>1</v>
       </c>
       <c r="I3" s="0">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.55">
-      <c r="A4" s="0">
-        <v>30003</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="0">
-        <v>100</v>
-      </c>
-      <c r="E4" s="0">
-        <v>100</v>
-      </c>
-      <c r="F4" s="0">
-        <v>10</v>
-      </c>
-      <c r="G4" s="0">
-        <v>5</v>
-      </c>
-      <c r="H4" s="0">
-        <v>1</v>
-      </c>
-      <c r="I4" s="0">
         <v>1</v>
       </c>
     </row>
@@ -815,7 +784,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="2" width="15.640625" customWidth="1"/>
@@ -828,7 +797,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C1" s="0" t="s">
         <v>1</v>
@@ -837,7 +806,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F1" s="0" t="s">
         <v>10</v>
@@ -853,14 +822,14 @@
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.55">
-      <c r="A2" s="0" t="s">
-        <v>29</v>
+      <c r="A2" s="0">
+        <v>40001</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="D2" s="0">
         <v>100</v>
@@ -872,41 +841,12 @@
         <v>5</v>
       </c>
       <c r="G2" s="0">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H2" s="0">
         <v>1</v>
       </c>
       <c r="I2" s="0">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.55">
-      <c r="A3" s="0">
-        <v>40002</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="0">
-        <v>100</v>
-      </c>
-      <c r="E3" s="0" t="b">
-        <v>0</v>
-      </c>
-      <c r="F3" s="0">
-        <v>5</v>
-      </c>
-      <c r="G3" s="0">
-        <v>1</v>
-      </c>
-      <c r="H3" s="0">
-        <v>1</v>
-      </c>
-      <c r="I3" s="0">
         <v>5</v>
       </c>
     </row>
@@ -918,10 +858,38 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.55">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.55">
+      <c r="A2" s="0">
+        <v>50001</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="0">
+        <v>180</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: AddTrainData, UpgradeTrainData 제작중
</commit_message>
<xml_diff>
--- a/Assets/TrainDefenseData.xlsx
+++ b/Assets/TrainDefenseData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chang\GitHub\TrainDefense\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{318DB933-A1C0-4B0E-86AF-ED5CD8D3B037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{076EC1A3-35C1-4121-9B06-17994D13ABB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5415" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5415" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="850" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monster_Data" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,9 @@
     <sheet name="Stage_Data" sheetId="3" r:id="rId5"/>
     <sheet name="Add_Train_Choice_Data" sheetId="6" r:id="rId6"/>
     <sheet name="Upgrade_Train_Choice_Data" sheetId="7" r:id="rId7"/>
+    <sheet name="Train_Upgrade_Data" sheetId="8" r:id="rId8"/>
+    <sheet name="Turret_Train_UpgradeData" sheetId="9" r:id="rId9"/>
+    <sheet name="Range_Train_Upgrade_Data" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="44">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -137,9 +140,6 @@
     <t>is_main_train</t>
   </si>
   <si>
-    <t>desc</t>
-  </si>
-  <si>
     <t>100</t>
   </si>
   <si>
@@ -159,10 +159,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Basic</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Slime</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -174,30 +170,45 @@
     <t>10;20;30</t>
   </si>
   <si>
-    <t>train_basic</t>
-  </si>
-  <si>
     <t>weight</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>choice_Type</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>train_Data_id</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>upgrade_data_id</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>upgrade_Data_Weight</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>target_Train_Id</t>
+    <t>train_data_id</t>
+  </si>
+  <si>
+    <t>target_train_id</t>
+  </si>
+  <si>
+    <t>기관총 포탑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>기관총으로 피해를 준다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>메인기차</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>제일 기본이 되는 기차이다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>냉기 포탑</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>범위 내에 있는 적들의 이동속도가 느려지고 피해를 준다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>weighted_upgrade_ids</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>upgrade_name</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -619,43 +630,103 @@
         <v>10001</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
         <v>21</v>
       </c>
       <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
         <v>25</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" t="s">
         <v>26</v>
       </c>
-      <c r="F2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" t="s">
         <v>27</v>
       </c>
-      <c r="H2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" t="s">
         <v>28</v>
-      </c>
-      <c r="J2" t="s">
-        <v>26</v>
-      </c>
-      <c r="K2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L2" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13BD03D1-5D02-4A2E-97F6-4C786BABBB78}">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="17.600000000000001" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="2" max="8" width="15.640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2">
+        <v>100001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3">
+        <v>100002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4">
+        <v>100003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5">
+        <v>100004</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -687,20 +758,20 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" t="s">
-        <v>35</v>
+      <c r="A2">
+        <v>20001</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="D2">
         <v>100</v>
       </c>
       <c r="E2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -712,7 +783,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="17.600000000000001" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="2" width="15.640625" customWidth="1"/>
@@ -754,28 +825,28 @@
         <v>30001</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="D2">
         <v>100</v>
       </c>
-      <c r="E2">
-        <v>100</v>
+      <c r="E2" t="b">
+        <v>0</v>
       </c>
       <c r="F2">
         <v>5</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
       <c r="I2">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.55000000000000004">
@@ -783,43 +854,73 @@
         <v>30002</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3">
         <v>100</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4">
+        <v>30003</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4">
         <v>100</v>
       </c>
-      <c r="F3">
+      <c r="E4" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4">
         <v>10</v>
       </c>
-      <c r="G3">
+      <c r="G4">
         <v>5</v>
       </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="17.600000000000001" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="2" width="15.640625" customWidth="1"/>
-    <col min="3" max="3" width="47.28515625" customWidth="1"/>
+    <col min="3" max="3" width="50.28515625" customWidth="1"/>
     <col min="4" max="13" width="15.640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -879,6 +980,35 @@
       </c>
       <c r="I2">
         <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3">
+        <v>40002</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D3">
+        <v>100</v>
+      </c>
+      <c r="E3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -901,10 +1031,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
@@ -912,7 +1042,7 @@
         <v>50001</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C2">
         <v>180</v>
@@ -926,38 +1056,82 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFFA9861-11E4-4B91-BB73-9FE61424E6A0}">
-  <dimension ref="A1:G1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="17.600000000000001" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="12.640625" customWidth="1"/>
     <col min="4" max="4" width="14.28515625" customWidth="1"/>
     <col min="5" max="5" width="16.92578125" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="13.92578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G1" t="s">
-        <v>41</v>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2">
+        <v>60001</v>
+      </c>
+      <c r="B2">
+        <v>30001</v>
+      </c>
+      <c r="C2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3">
+        <v>60002</v>
+      </c>
+      <c r="B3">
+        <v>30002</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4">
+        <v>60003</v>
+      </c>
+      <c r="B4">
+        <v>30003</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5">
+        <v>60004</v>
+      </c>
+      <c r="B5">
+        <v>40001</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6">
+        <v>60005</v>
+      </c>
+      <c r="B6">
+        <v>40002</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -968,12 +1142,13 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{944099CA-CBCA-415A-AFA2-2DF61D5E4CE1}">
-  <dimension ref="A1:E1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="17.600000000000001" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="21.28515625" customWidth="1"/>
+    <col min="2" max="2" width="13.92578125" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" customWidth="1"/>
     <col min="5" max="5" width="13.78515625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -982,16 +1157,184 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E1" t="s">
-        <v>41</v>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2">
+        <v>70001</v>
+      </c>
+      <c r="B2">
+        <v>30001</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3">
+        <v>70002</v>
+      </c>
+      <c r="B3">
+        <v>30002</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4">
+        <v>70003</v>
+      </c>
+      <c r="B4">
+        <v>30003</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5">
+        <v>70004</v>
+      </c>
+      <c r="B5">
+        <v>40001</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6">
+        <v>70005</v>
+      </c>
+      <c r="B6">
+        <v>40002</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84517C9E-E38E-4A09-A50B-E00504ACBE9C}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="17.600000000000001" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2">
+        <v>80001</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24E50DA9-A70A-4558-8529-6E6BDC7C52F5}">
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr defaultRowHeight="17.600000000000001" x14ac:dyDescent="0.55000000000000004"/>
+  <cols>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" customWidth="1"/>
+    <col min="8" max="8" width="15.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2">
+        <v>90001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3">
+        <v>90002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4">
+        <v>90003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5">
+        <v>90004</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6">
+        <v>90005</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7">
+        <v>90006</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Upgrade 제작 완료
</commit_message>
<xml_diff>
--- a/Assets/TrainDefenseData.xlsx
+++ b/Assets/TrainDefenseData.xlsx
@@ -1,30 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="HCell" lastEdited="11.0" lowestEdited="11.0" rupBuild="0.2292"/>
-  <workbookPr codeName="ThisWorkbook" autoCompressPictures="1"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="28545" windowHeight="11700" tabRatio="839" firstSheet="2" activeTab="2"/>
+    <workbookView xWindow="5415" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="839" firstSheet="2" activeTab="5"/>
   </bookViews>
   <sheets>
-    <sheet name="Monster_Data" sheetId="1" r:id="rId4"/>
-    <sheet name="Train_Data" sheetId="2" r:id="rId5"/>
-    <sheet name="Turret_Train_Data" sheetId="3" r:id="rId6"/>
-    <sheet name="Range_Train_Data" sheetId="4" r:id="rId7"/>
-    <sheet name="Stage_Data" sheetId="5" r:id="rId8"/>
-    <sheet name="Add_Train_Choice_Data" sheetId="6" r:id="rId9"/>
-    <sheet name="Upgrade_Train_Choice_Data" sheetId="7" r:id="rId10"/>
-    <sheet name="Train_Upgrade_Data" sheetId="8" r:id="rId11"/>
-    <sheet name="Turret_Train_Upgrade_Data" sheetId="9" r:id="rId12"/>
-    <sheet name="Range_Train_Upgrade_Data" sheetId="10" r:id="rId13"/>
-    <sheet name="Upgrade_Data" sheetId="11" r:id="rId14"/>
+    <sheet name="Monster_Data" sheetId="1" r:id="rId1"/>
+    <sheet name="Train_Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Range_Train_Data" sheetId="4" r:id="rId3"/>
+    <sheet name="Turret_Train_Data" sheetId="3" r:id="rId4"/>
+    <sheet name="Stage_Data" sheetId="5" r:id="rId5"/>
+    <sheet name="Add_Train_Choice_Data" sheetId="6" r:id="rId6"/>
+    <sheet name="Upgrade_Train_Choice_Data" sheetId="7" r:id="rId7"/>
+    <sheet name="Train_Upgrade_Data" sheetId="8" r:id="rId8"/>
+    <sheet name="Turret_Train_Upgrade_Data" sheetId="9" r:id="rId9"/>
+    <sheet name="Range_Train_Upgrade_Data" sheetId="10" r:id="rId10"/>
+    <sheet name="Upgrade_Data" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr/>
+  <fileRecoveryPr autoRecover="0" crashSave="0" dataExtractLoad="0" repairLoad="0"/>
+  <extLst>
+    <ext uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="99">
   <si>
     <t xml:space="preserve">포탑들의 공격 딜레이가 {0}({1})만큼 감소합니다.</t>
   </si>
@@ -300,6 +306,34 @@
   </si>
   <si>
     <t xml:space="preserve">FireEffectProjectile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">upgrade_type</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">NonTrainUpgrade</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">TrainUpgrade</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">stat_type</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">MaxHp</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">AttackDamage</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">AttackInterval</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -307,7 +341,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -317,26 +351,14 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="맑은 고딕"/>
+      <sz val="8"/>
+      <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
     </font>
   </fonts>
   <fills count="2">
@@ -349,18 +371,11 @@
   </fills>
   <borders count="1">
     <border>
-      <left>
-        <color indexed="64"/>
-      </left>
-      <right>
-        <color indexed="64"/>
-      </right>
-      <top>
-        <color indexed="64"/>
-      </top>
-      <bottom>
-        <color indexed="64"/>
-      </bottom>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -368,42 +383,28 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf/>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFAEBFEA"/>
-          <bgColor rgb="FFAEBFEA"/>
+          <fgColor rgb="FF6182D6"/>
+          <bgColor rgb="FF6182D6"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF94A5DF"/>
-          <bgColor rgb="FF94A5DF"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color rgb="FF6182D6"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF6182D6"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <fill>
@@ -415,28 +416,20 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Normal Style 1 - Accent 1" pivot="0" table="1" count="9">
-      <tableStyleElement type="wholeTable" size="1"/>
-      <tableStyleElement type="headerRow" size="1" dxfId="5"/>
-      <tableStyleElement type="totalRow" size="1" dxfId="4"/>
-      <tableStyleElement type="firstColumn" size="1" dxfId="3"/>
-      <tableStyleElement type="lastColumn" size="1" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" size="1" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" size="1" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" size="1" dxfId="2"/>
-      <tableStyleElement type="secondColumnStripe" size="1" dxfId="1"/>
+    <tableStyle name="Normal Style 1 - Accent 1" pivot="0" table="0" count="2">
+      <tableStyleElement type="firstColumn" dxfId="1"/>
+      <tableStyleElement type="lastColumn"/>
     </tableStyle>
-    <tableStyle name="Light Style 1 - Accent 1" pivot="1" table="0" count="8">
-      <tableStyleElement type="wholeTable" size="1" dxfId="6"/>
-      <tableStyleElement type="headerRow" size="1" dxfId="11"/>
-      <tableStyleElement type="totalRow" size="1" dxfId="10"/>
-      <tableStyleElement type="firstColumn" size="1" dxfId="9"/>
-      <tableStyleElement type="lastColumn" size="1" dxfId="9"/>
-      <tableStyleElement type="firstRowStripe" size="1" dxfId="7"/>
-      <tableStyleElement type="secondRowStripe" size="1" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" size="1" dxfId="8"/>
-    </tableStyle>
+    <tableStyle name="Light Style 1 - Accent 1" pivot="0" table="0"/>
   </tableStyles>
+  <extLst>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -725,6 +718,8 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -732,7 +727,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:N2"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="17.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="2" max="2" width="15.5" style="1" customWidth="1"/>
     <col min="3" max="3" width="22.5703125" style="1" customWidth="1"/>
@@ -746,7 +741,7 @@
     <col min="13" max="13" width="11.85546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
@@ -787,7 +782,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A2" s="1">
         <v>10001</v>
       </c>
@@ -829,8 +824,9 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -838,7 +834,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:J3"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="17.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="2" max="2" width="15.640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="27.5" style="1" customWidth="1"/>
@@ -846,7 +842,7 @@
     <col min="9" max="9" width="19.78515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
@@ -875,7 +871,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A2" s="1">
         <v>100001</v>
       </c>
@@ -892,7 +888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A3" s="1">
         <v>100002</v>
       </c>
@@ -910,6 +906,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
 </worksheet>
@@ -918,8 +915,8 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet11"/>
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="17.6"/>
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="2" max="2" width="21.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="48.5703125" style="1" customWidth="1"/>
@@ -927,9 +924,11 @@
     <col min="5" max="5" width="15.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="18.78515625" style="1" customWidth="1"/>
     <col min="7" max="7" width="12.78515625" style="1" customWidth="1"/>
+    <col min="8" max="9" width="19.35546875" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
@@ -951,8 +950,15 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="H1" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A2" s="1">
         <v>110001</v>
       </c>
@@ -971,8 +977,14 @@
       <c r="F2" s="1">
         <v>100</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="H2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A3" s="1">
         <v>110002</v>
       </c>
@@ -986,13 +998,19 @@
         <v>200</v>
       </c>
       <c r="E3" s="1">
-        <v>-0.10000000000000001</v>
+        <v>-0.1</v>
       </c>
       <c r="F3" s="1">
         <v>100</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="H3" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A4" s="1">
         <v>110003</v>
       </c>
@@ -1011,8 +1029,14 @@
       <c r="F4" s="1">
         <v>50</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="H4" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A5" s="1">
         <v>110004</v>
       </c>
@@ -1031,8 +1055,11 @@
       <c r="F5" s="1">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="H5" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.55">
       <c r="A6" s="1">
         <v>110005</v>
       </c>
@@ -1051,10 +1078,14 @@
       <c r="F6" s="1">
         <v>10</v>
       </c>
+      <c r="H6" s="2" t="s">
+        <v>93</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1062,14 +1093,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="17.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="2" width="15.640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="46.28515625" style="1" customWidth="1"/>
     <col min="4" max="13" width="15.640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
@@ -1092,7 +1123,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.55">
       <c r="A2" s="1">
         <v>20001</v>
       </c>
@@ -1113,6 +1144,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -1120,9 +1152,140 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr codeName="Sheet4"/>
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
+  <cols>
+    <col min="1" max="2" width="15.640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="50.28515625" style="1" customWidth="1"/>
+    <col min="4" max="5" width="15.640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="19.140625" style="1" customWidth="1"/>
+    <col min="7" max="10" width="15.640625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.2109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="21" style="1" customWidth="1"/>
+    <col min="13" max="13" width="15.640625" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.55">
+      <c r="A1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.55">
+      <c r="A2" s="1">
+        <v>40001</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="1">
+        <v>100</v>
+      </c>
+      <c r="E2" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H2" s="1">
+        <v>5</v>
+      </c>
+      <c r="I2" s="1">
+        <v>5</v>
+      </c>
+      <c r="J2" s="1">
+        <v>1</v>
+      </c>
+      <c r="K2" s="1">
+        <v>5</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.55">
+      <c r="A3" s="1">
+        <v>40002</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1">
+        <v>100</v>
+      </c>
+      <c r="E3" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="H3" s="1">
+        <v>5</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1</v>
+      </c>
+      <c r="J3" s="1">
+        <v>1</v>
+      </c>
+      <c r="K3" s="1">
+        <v>1</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:N8"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="2" width="15.640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="47.92578125" style="1" customWidth="1"/>
@@ -1134,7 +1297,7 @@
     <col min="13" max="13" width="15.640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
@@ -1165,8 +1328,8 @@
       <c r="J1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>38</v>
+      <c r="K1" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>44</v>
@@ -1175,7 +1338,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A2" s="1">
         <v>30001</v>
       </c>
@@ -1204,7 +1367,7 @@
         <v>1</v>
       </c>
       <c r="K2" s="1">
-        <v>0.29999999999999999</v>
+        <v>0.3</v>
       </c>
       <c r="L2" s="1">
         <v>0</v>
@@ -1213,7 +1376,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A3" s="1">
         <v>30002</v>
       </c>
@@ -1242,7 +1405,7 @@
         <v>1</v>
       </c>
       <c r="K3" s="1">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="L3" s="1">
         <v>0</v>
@@ -1251,7 +1414,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A4" s="1">
         <v>30003</v>
       </c>
@@ -1289,7 +1452,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A5" s="1">
         <v>30004</v>
       </c>
@@ -1327,7 +1490,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A6" s="1">
         <v>30005</v>
       </c>
@@ -1365,7 +1528,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A7" s="1">
         <v>30006</v>
       </c>
@@ -1403,7 +1566,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.55">
       <c r="A8" s="1">
         <v>30007</v>
       </c>
@@ -1432,7 +1595,7 @@
         <v>1</v>
       </c>
       <c r="K8" s="1">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L8" s="1">
         <v>0</v>
@@ -1442,138 +1605,9 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <sheetPr codeName="Sheet4"/>
-  <dimension ref="A1:M3"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="17.6"/>
-  <cols>
-    <col min="1" max="2" width="15.640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="50.28515625" style="1" customWidth="1"/>
-    <col min="4" max="5" width="15.640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.140625" style="1" customWidth="1"/>
-    <col min="7" max="10" width="15.640625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="18.2109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="21" style="1" customWidth="1"/>
-    <col min="13" max="13" width="15.640625" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:12">
-      <c r="A1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12">
-      <c r="A2" s="1">
-        <v>40001</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D2" s="1">
-        <v>100</v>
-      </c>
-      <c r="E2" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="H2" s="1">
-        <v>5</v>
-      </c>
-      <c r="I2" s="1">
-        <v>5</v>
-      </c>
-      <c r="J2" s="1">
-        <v>1</v>
-      </c>
-      <c r="K2" s="1">
-        <v>5</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="A3" s="1">
-        <v>40002</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" s="1">
-        <v>100</v>
-      </c>
-      <c r="E3" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="H3" s="1">
-        <v>5</v>
-      </c>
-      <c r="I3" s="1">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1">
-        <v>1</v>
-      </c>
-      <c r="K3" s="1">
-        <v>1</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
-  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1581,13 +1615,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="17.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="2" max="2" width="21.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="14.5" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
@@ -1598,7 +1632,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A2" s="1">
         <v>50001</v>
       </c>
@@ -1610,6 +1644,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -1619,7 +1654,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="16.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="2" max="2" width="12" style="1" customWidth="1"/>
     <col min="3" max="3" width="12.640625" style="1" customWidth="1"/>
@@ -1629,7 +1664,7 @@
     <col min="7" max="7" width="13.92578125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
@@ -1640,7 +1675,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A2" s="1">
         <v>60001</v>
       </c>
@@ -1648,10 +1683,10 @@
         <v>30001</v>
       </c>
       <c r="C2" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A3" s="1">
         <v>60002</v>
       </c>
@@ -1662,7 +1697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A4" s="1">
         <v>60003</v>
       </c>
@@ -1673,7 +1708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A5" s="1">
         <v>60004</v>
       </c>
@@ -1684,7 +1719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A6" s="1">
         <v>60005</v>
       </c>
@@ -1695,7 +1730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A7" s="1">
         <v>60006</v>
       </c>
@@ -1706,7 +1741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A8" s="1">
         <v>60007</v>
       </c>
@@ -1714,10 +1749,10 @@
         <v>30007</v>
       </c>
       <c r="C8" s="1">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A9" s="1">
         <v>60008</v>
       </c>
@@ -1728,7 +1763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.55">
       <c r="A10" s="1">
         <v>60009</v>
       </c>
@@ -1740,8 +1775,9 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1749,7 +1785,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="17.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="2" max="2" width="13.92578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="26.85546875" style="1" customWidth="1"/>
@@ -1757,7 +1793,7 @@
     <col min="5" max="5" width="13.78515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
@@ -1774,7 +1810,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A2" s="1">
         <v>70001</v>
       </c>
@@ -1791,7 +1827,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A3" s="1">
         <v>70002</v>
       </c>
@@ -1808,7 +1844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A4" s="1">
         <v>70003</v>
       </c>
@@ -1825,7 +1861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A5" s="1">
         <v>70004</v>
       </c>
@@ -1842,7 +1878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A6" s="1">
         <v>70005</v>
       </c>
@@ -1860,6 +1896,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
 </worksheet>
@@ -1869,13 +1906,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="17.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="1" max="1" width="15.78515625" style="1" customWidth="1"/>
     <col min="2" max="2" width="13.5" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
@@ -1892,12 +1929,13 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.55">
       <c r="A2" s="1">
         <v>80001</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
@@ -1907,7 +1945,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultColWidth="9.00390625" defaultRowHeight="17.6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.6" x14ac:dyDescent="0.55"/>
   <cols>
     <col min="2" max="2" width="14.28515625" style="1" customWidth="1"/>
     <col min="3" max="3" width="32.42578125" style="1" customWidth="1"/>
@@ -1919,7 +1957,7 @@
     <col min="9" max="9" width="16" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
@@ -1944,11 +1982,11 @@
       <c r="H1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="I1" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A2" s="1">
         <v>90001</v>
       </c>
@@ -1962,10 +2000,10 @@
         <v>1</v>
       </c>
       <c r="I2" s="1">
-        <v>0.10000000000000001</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A3" s="1">
         <v>90002</v>
       </c>
@@ -1979,7 +2017,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.55">
       <c r="A4" s="1">
         <v>90003</v>
       </c>
@@ -1993,10 +2031,11 @@
         <v>1</v>
       </c>
       <c r="I4" s="1">
-        <v>0.10000000000000001</v>
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
   <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Train 죽음 & 부활 제작
</commit_message>
<xml_diff>
--- a/Assets/TrainDefenseData.xlsx
+++ b/Assets/TrainDefenseData.xlsx
@@ -903,7 +903,7 @@
         <v>100001</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>83</v>
@@ -912,7 +912,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="1">
-        <v>1</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.55">
@@ -920,7 +920,7 @@
         <v>100001</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>96</v>
@@ -929,7 +929,7 @@
         <v>1</v>
       </c>
       <c r="G3" s="1">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.55">
@@ -937,7 +937,7 @@
         <v>100001</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>83</v>
@@ -946,7 +946,7 @@
         <v>1</v>
       </c>
       <c r="G4" s="1">
-        <v>2</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.55">
@@ -954,7 +954,7 @@
         <v>100002</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>83</v>
@@ -963,7 +963,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="1">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="I5" s="2"/>
     </row>
@@ -972,7 +972,7 @@
         <v>100002</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>83</v>
@@ -981,7 +981,7 @@
         <v>1</v>
       </c>
       <c r="G6" s="1">
-        <v>100</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.55">
@@ -989,7 +989,7 @@
         <v>100002</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>83</v>
@@ -998,13 +998,13 @@
         <v>1</v>
       </c>
       <c r="G7" s="1">
-        <v>250</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.699861109256744" right="0.699861109256744" top="0.75" bottom="0.75" header="0.300000011920929" footer="0.300000011920929"/>
-  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>